<commit_message>
Update: improved browser actions and automation
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -413,34 +413,74 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Priority</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Item 1</t>
+          <t>Draft plan</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Item 2</t>
+          <t>Run tests</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Item 3</t>
+          <t>Write summary</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>

</xml_diff>